<commit_message>
corrige tab2 : retrait du corrige cache
</commit_message>
<xml_diff>
--- a/contenus/tab2/exs1-recherchev-prix.xlsx
+++ b/contenus/tab2/exs1-recherchev-prix.xlsx
@@ -9,7 +9,6 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consignes" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercice" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Correction" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1011,380 +1010,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Référence</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Quantité commandée</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Prix unitaire (€)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>REF003</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>3</v>
-      </c>
-      <c r="C2">
-        <f>VLOOKUP(A2,$F$2:$H$16,3,FALSE)</f>
-        <v/>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>REF001</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Casque de chantier</t>
-        </is>
-      </c>
-      <c r="H2" t="n">
-        <v>12.5</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>REF008</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C3">
-        <f>VLOOKUP(A3,$F$2:$H$16,3,FALSE)</f>
-        <v/>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>REF002</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Gants de manutention</t>
-        </is>
-      </c>
-      <c r="H3" t="n">
-        <v>4.2</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>REF001</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>20</v>
-      </c>
-      <c r="C4">
-        <f>VLOOKUP(A4,$F$2:$H$16,3,FALSE)</f>
-        <v/>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>REF003</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Chaussures de sécurité</t>
-        </is>
-      </c>
-      <c r="H4" t="n">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>REF012</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>15</v>
-      </c>
-      <c r="C5">
-        <f>VLOOKUP(A5,$F$2:$H$16,3,FALSE)</f>
-        <v/>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>REF004</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Gilet haute visibilité</t>
-        </is>
-      </c>
-      <c r="H5" t="n">
-        <v>8.9</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>REF005</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>25</v>
-      </c>
-      <c r="C6">
-        <f>VLOOKUP(A6,$F$2:$H$16,3,FALSE)</f>
-        <v/>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>REF005</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Lunettes de protection</t>
-        </is>
-      </c>
-      <c r="H6" t="n">
-        <v>6.5</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>REF014</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7">
-        <f>VLOOKUP(A7,$F$2:$H$16,3,FALSE)</f>
-        <v/>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>REF006</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Bouchons d'oreille (boîte)</t>
-        </is>
-      </c>
-      <c r="H7" t="n">
-        <v>3.2</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>REF002</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>40</v>
-      </c>
-      <c r="C8">
-        <f>VLOOKUP(A8,$F$2:$H$16,3,FALSE)</f>
-        <v/>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>REF007</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Diable pliant</t>
-        </is>
-      </c>
-      <c r="H8" t="n">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>REF010</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>8</v>
-      </c>
-      <c r="C9">
-        <f>VLOOKUP(A9,$F$2:$H$16,3,FALSE)</f>
-        <v/>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>REF008</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Transpalette manuel</t>
-        </is>
-      </c>
-      <c r="H9" t="n">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>REF007</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>2</v>
-      </c>
-      <c r="C10">
-        <f>VLOOKUP(A10,$F$2:$H$16,3,FALSE)</f>
-        <v/>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>REF009</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Rouleau de film étirable</t>
-        </is>
-      </c>
-      <c r="H10" t="n">
-        <v>15.8</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>REF013</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>10</v>
-      </c>
-      <c r="C11">
-        <f>VLOOKUP(A11,$F$2:$H$16,3,FALSE)</f>
-        <v/>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>REF010</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Carton d'emballage (lot de 20)</t>
-        </is>
-      </c>
-      <c r="H11" t="n">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>REF011</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Étiquettes code-barres (rouleau)</t>
-        </is>
-      </c>
-      <c r="H12" t="n">
-        <v>9.9</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>REF012</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Sangle d'arrimage</t>
-        </is>
-      </c>
-      <c r="H13" t="n">
-        <v>11.4</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>REF013</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Cadenas de sécurité</t>
-        </is>
-      </c>
-      <c r="H14" t="n">
-        <v>7.6</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>REF014</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Chariot de manutention</t>
-        </is>
-      </c>
-      <c r="H15" t="n">
-        <v>620</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>REF015</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Extincteur portatif</t>
-        </is>
-      </c>
-      <c r="H16" t="n">
-        <v>65</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>